<commit_message>
[2026.08.09] 엑셀 시트 수정
- 내러티브, 시스템 시트 수정 (불필요한 퀘스트 플로우 삭제)
</commit_message>
<xml_diff>
--- a/Document/데이터/LUNA_System.xlsx
+++ b/Document/데이터/LUNA_System.xlsx
@@ -9,25 +9,27 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INFO" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cocktails" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecipeLines" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShelfItems" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personalities" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RandomWaves" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GradeCuts" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GradePayout" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuestBodies" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tags" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecipeLines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShelfItems" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personalities" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RandomWaves" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GradeCuts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GradePayout" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuestBodies" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cocktails'!$A$1:$V$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RecipeLines'!$A$1:$F$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ShelfItems'!$A$1:$L$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Personalities'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'RandomWaves'!$A$1:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Config'!$A$1:$D$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'GradeCuts'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'GradePayout'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'GuestBodies'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cocktails'!$A$1:$Z$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tags'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RecipeLines'!$A$1:$F$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ShelfItems'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Personalities'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'RandomWaves'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Config'!$A$1:$D$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'GradeCuts'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'GradePayout'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'GuestBodies'!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -313,17 +315,13 @@
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>[자동 계산 컬럼]
-빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
-계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+        <t>제조법 설명(한국어) — 정보 화면과 레시피 팝업에 그대로 뜨는 문장. 손으로 적는다. RecipeLines는 채점 정답표이고 이 칸은 표시 전용이라, 수치를 고치면 이 문장도 같이 고쳐야 한다
 💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>[자동 계산 컬럼]
-빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
-계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+        <t>제조법 설명(영어)
 💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
       </text>
     </comment>
@@ -351,11 +349,147 @@
 💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
       </text>
     </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>[자동 계산 컬럼]
+빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
+계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>[자동 계산 컬럼]
+빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
+계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>[자동 계산 컬럼]
+빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
+계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>[자동 계산 컬럼]
+빌드가 값을 채우는 칸이다. 손으로 고쳐도 다음 빌드에서 덮어써진다.
+계산 근거를 바꾸고 싶으면 재료·레시피·override 컬럼을 수정할 것.
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>LUNA 데이터 가이드</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>📋 [GuestBodies 시트]
+랜덤 손님 공용 외형 카탈로그 — 바디(얼굴·코·입 포함)×의상×눈×헤어를 성별 맞춰 조합. 스폰 시 성별 추첨 후, 그 손님 성격을 허용하는 항목만 남겨 파트별 weight 가중 랜덤
+── 이 컬럼 ──
+파트 종류 — body(바디: 얼굴·몸통·코·입·패널 라인 한 장)/outfit(의상)/eyes(눈)/hair(헤어). 스폰 시 파트별로 하나씩 추첨해 겹쳐 그린다(바디→의상→눈→헤어 순)
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>snake_case 고유 id
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>m/f — 같은 성별 파트끼리만 조합된다
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>이 파트를 쓸 수 있는 성격 — 세미콜론 구분(예: rough;touchy). 비우면 전 성격 공용. 성격별 전용 외형을 만들 때 채운다
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>sprite=이미지 한 장(현행) / parts_anim=파츠 애니(추후 전환용 — 단골 표정과 같은 규칙)
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>sprite 모드의 리소스 키. 아트 제작 중이라 지금은 가칭 — 완성 시 실키로 교체
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>표정별 교체 스프라이트 — '표정:키; 표정:키' (예: joy:Guest/eyes_m_1_joy; anger:…). 표정이 정해지면 이 맵에 있는 표정만 교체, 없으면 기본 sprite 유지. 비우면 표정 고정(현행). 표정은 common 세트, default 등록 금지. 감정 눈 아트가 나오면 eyes 행에 채운다
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>추첨 가중치(1 이상 정수). 클수록 자주 나온다
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>제작중/OK — 에셋 검수용, 게임 미사용
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>기획 메모 (게임 미사용)
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>LUNA 데이터 가이드</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>📋 [Tags 시트]
+맛 키워드 사전. 칵테일 tags와 Tastes의 cocktail.tag(...)이 여기 적힌 한글 태그만 쓸 수 있고, 영어 표기는 정보 화면 키워드 표시에 쓰인다
+── 이 컬럼 ──
+태그 한글 표기(정본 키). Cocktails.tags와 Tastes의 cocktail.tag(...)이 이 값을 그대로 쓴다
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>영어 표기 — 정보 화면 키워드가 EN 빌드에서 이 값을 표시
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>작업 메모
+💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -404,7 +538,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -489,7 +623,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -544,7 +678,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -599,7 +733,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -636,7 +770,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -661,7 +795,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>LUNA 데이터 가이드</author>
@@ -679,79 +813,6 @@
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>술값 배율. 1.0=정가 다 받음, **음수면 배상**(-1.0 = 술값만큼 물어줌). sewage와 오제조만 음수
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>LUNA 데이터 가이드</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>📋 [GuestBodies 시트]
-랜덤 손님 공용 외형 카탈로그 — 바디(얼굴·코·입 포함)×의상×눈×헤어를 성별 맞춰 조합. 스폰 시 성별 추첨 후, 그 손님 성격을 허용하는 항목만 남겨 파트별 weight 가중 랜덤
-── 이 컬럼 ──
-파트 종류 — body(바디: 얼굴·몸통·코·입·패널 라인 한 장)/outfit(의상)/eyes(눈)/hair(헤어). 스폰 시 파트별로 하나씩 추첨해 겹쳐 그린다(바디→의상→눈→헤어 순)
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>snake_case 고유 id
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>m/f — 같은 성별 파트끼리만 조합된다
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>이 파트를 쓸 수 있는 성격 — 세미콜론 구분(예: rough;touchy). 비우면 전 성격 공용. 성격별 전용 외형을 만들 때 채운다
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>sprite=이미지 한 장(현행) / parts_anim=파츠 애니(추후 전환용 — 단골 표정과 같은 규칙)
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>sprite 모드의 리소스 키. 아트 제작 중이라 지금은 가칭 — 완성 시 실키로 교체
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>표정별 교체 스프라이트 — '표정:키; 표정:키' (예: joy:Guest/eyes_m_1_joy; anger:…). 표정이 정해지면 이 맵에 있는 표정만 교체, 없으면 기본 sprite 유지. 비우면 표정 고정(현행). 표정은 common 세트, default 등록 금지. 감정 눈 아트가 나오면 eyes 행에 채운다
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>추첨 가중치(1 이상 정수). 클수록 자주 나온다
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>제작중/OK — 에셋 검수용, 게임 미사용
-💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>기획 메모 (게임 미사용)
 💡 헤더에 마우스를 올리면 이 설명이 보입니다.</t>
       </text>
     </comment>
@@ -1391,6 +1452,89 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00ED7D31"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>grade</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>revenue_mult</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>decent</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sewage</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2032,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2052,11 +2196,15 @@
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2145,29 +2293,49 @@
           <t>tier_override</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>recipe_desc_ko</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>recipe_desc_en</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>(파생)tier</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>(파생)gimmick</t>
         </is>
       </c>
-      <c r="T1" s="5" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>(파생)unlock_day</t>
         </is>
       </c>
-      <c r="U1" s="5" t="inlineStr">
+      <c r="W1" s="5" t="inlineStr">
         <is>
           <t>(파생)scoring_items</t>
         </is>
       </c>
-      <c r="V1" s="5" t="inlineStr">
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>(파생)time_limit</t>
+        </is>
+      </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>(파생)sprite</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>(파생)serve_sprite</t>
         </is>
       </c>
     </row>
@@ -2237,22 +2405,42 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>하이볼 잔에 진 1.5oz를 붓고, 토닉워터로 잔을 채워 가볍게 젓는다. 라임 웨지를 걸친다.</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>Pour 1.5oz gin into a highball glass, top with tonic water, and stir gently. Garnish with a lime wedge.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>2</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>1</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>6</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>36</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Finished_GinTonic</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Serve_GinTonic</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -2321,22 +2509,42 @@
       <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr"/>
       <c r="Q3" s="7" t="inlineStr"/>
-      <c r="R3" s="7" t="inlineStr">
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>진 1.5oz, 레몬 반 개의 즙, 설탕 1tsp을 셰이킹해 하이볼 잔에 따른다. 소다수로 채우고 레몬 슬라이스를 올린다.</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Shake 1.5oz gin, the juice of half a lemon, and 1 tsp sugar, then strain into a highball glass. Top with soda water and add a lemon slice.</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S3" s="7" t="n">
+      <c r="U3" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="T3" s="7" t="n">
+      <c r="V3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="U3" s="7" t="n">
+      <c r="W3" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="V3" s="7" t="n">
+      <c r="X3" s="7" t="n">
         <v>52</v>
+      </c>
+      <c r="Y3" s="7" t="inlineStr">
+        <is>
+          <t>Finished_GinFizz</t>
+        </is>
+      </c>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>Serve_GinFizz</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -2401,22 +2609,42 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>오프너로 뚜껑을 딴 뒤 맥주잔에 12oz를 천천히 따른다. 거품이 잔 위로 넘치지 않게 기울여서.</t>
+        </is>
+      </c>
+      <c r="S4" s="6" t="inlineStr">
+        <is>
+          <t>Pop the cap with an opener and pour 12oz slowly into a beer mug, tilted so the head doesn't spill over.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>2</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>1</v>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>5</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>36</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Finished_BottleBeer</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Serve_BottleBeer</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -2481,22 +2709,42 @@
       <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="7" t="inlineStr"/>
       <c r="Q5" s="7" t="inlineStr"/>
-      <c r="R5" s="7" t="inlineStr">
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>코르크를 조심스럽게 뽑고 와인잔에 8oz를 따른다. 잔을 흔들지 않는다.</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>Draw the cork carefully and pour 8oz into a wine glass. Do not swirl.</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="S5" s="7" t="n">
+      <c r="U5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="T5" s="7" t="n">
+      <c r="V5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="U5" s="7" t="n">
+      <c r="W5" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="V5" s="7" t="n">
+      <c r="X5" s="7" t="n">
         <v>36</v>
+      </c>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>Finished_RedWine</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>Serve_RedWine</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2561,22 +2809,42 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>코르크를 소리 없이 뽑고 플루트 잔에 8oz를 따른다. 기포가 가라앉기 전에 낸다.</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>Ease the cork out without a pop and pour 8oz into a flute. Serve before the bubbles settle.</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>2</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>1</v>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>36</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Finished_Champagne</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Serve_Champagne</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2637,22 +2905,42 @@
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr"/>
       <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr">
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>하이볼 잔에 보드카 1.5oz와 오렌지주스 6oz를 넣고 젓는다.</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>Build 1.5oz vodka and 6oz orange juice in a highball glass and stir.</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="S7" s="7" t="n">
+      <c r="U7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="T7" s="7" t="n">
+      <c r="V7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="U7" s="7" t="n">
+      <c r="W7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="V7" s="7" t="n">
+      <c r="X7" s="7" t="n">
         <v>44</v>
+      </c>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>Finished_Screwdriver</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t>Serve_Screwdriver</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2721,22 +3009,42 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>맥주잔에 보드카 1.5oz와 라임 반 개의 즙을 넣고 젓는다. 진저에일로 채우고 라임 웨지를 걸친다.</t>
+        </is>
+      </c>
+      <c r="S8" s="6" t="inlineStr">
+        <is>
+          <t>Build 1.5oz vodka and the juice of half a lime in a mug and stir. Top with ginger ale and garnish with a lime wedge.</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>3</v>
       </c>
-      <c r="T8" t="n">
+      <c r="V8" t="n">
         <v>3</v>
       </c>
-      <c r="U8" t="n">
+      <c r="W8" t="n">
         <v>7</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>44</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Finished_MoscowMule</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Serve_MoscowMule</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2801,22 +3109,42 @@
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr"/>
       <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr">
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>콜린스 잔에 데킬라 1oz와 오렌지주스 6oz를 넣고 젓는다. 오렌지 슬라이스를 올린다.</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>Build 1oz tequila and 6oz orange juice in a collins glass and stir. Garnish with an orange slice.</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="S9" s="7" t="n">
+      <c r="U9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="T9" s="7" t="n">
+      <c r="V9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="U9" s="7" t="n">
+      <c r="W9" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="V9" s="7" t="n">
+      <c r="X9" s="7" t="n">
         <v>44</v>
+      </c>
+      <c r="Y9" s="7" t="inlineStr">
+        <is>
+          <t>Finished_TequilaSunrise</t>
+        </is>
+      </c>
+      <c r="Z9" s="7" t="inlineStr">
+        <is>
+          <t>Serve_TequilaSunrise</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2885,22 +3213,42 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>콜린스 잔에 진·보드카·럼·데킬라를 1oz씩 넣고 라임 반 개의 즙을 더해 젓는다. 콜라로 채우고 레몬 슬라이스를 올린다.</t>
+        </is>
+      </c>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>Build 1oz each of gin, vodka, rum, and tequila in a collins glass, add the juice of half a lime, and stir. Top with cola and add a lemon slice.</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>6</v>
       </c>
-      <c r="T10" t="n">
+      <c r="V10" t="n">
         <v>3</v>
       </c>
-      <c r="U10" t="n">
+      <c r="W10" t="n">
         <v>10</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>68</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Finished_LongIsland</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Serve_LongIsland</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -2969,22 +3317,42 @@
       <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr"/>
       <c r="Q11" s="7" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr">
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>위스키 1.5oz, 레몬 반 개의 즙, 설탕 1tsp을 셰이킹해 온더락 잔에 따른다. 사워믹스로 채우고 체리를 올린다.</t>
+        </is>
+      </c>
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>Shake 1.5oz whiskey, the juice of half a lemon, and 1 tsp sugar, then strain into a rocks glass. Top with sour mix and garnish with a cherry.</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S11" s="7" t="n">
+      <c r="U11" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="T11" s="7" t="n">
+      <c r="V11" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="U11" s="7" t="n">
+      <c r="W11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="V11" s="7" t="n">
+      <c r="X11" s="7" t="n">
         <v>52</v>
+      </c>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>Finished_WhiskeySour</t>
+        </is>
+      </c>
+      <c r="Z11" s="7" t="inlineStr">
+        <is>
+          <t>Serve_WhiskeySour</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3049,22 +3417,42 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>믹싱 글라스에 진 6oz와 드라이 버무스 1.5oz를 넣고 스터한 뒤 칵테일 잔에 따른다. 올리브를 넣는다.</t>
+        </is>
+      </c>
+      <c r="S12" s="6" t="inlineStr">
+        <is>
+          <t>Stir 6oz gin with 1.5oz dry vermouth in a mixing glass, then strain into a cocktail glass. Drop in an olive.</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>3</v>
       </c>
-      <c r="T12" t="n">
+      <c r="V12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="n">
+      <c r="W12" t="n">
         <v>6</v>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
         <v>44</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Finished_DryMartini</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Serve_DryMartini</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3125,22 +3513,42 @@
       <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr"/>
       <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr">
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>럼 4.5oz, 그레나딘 0.75oz, 라임즙 1.5oz를 셰이킹해 칵테일 잔에 따른다.</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>Shake 4.5oz rum, 0.75oz grenadine, and 1.5oz lime juice, then strain into a cocktail glass.</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S13" s="7" t="n">
+      <c r="U13" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="T13" s="7" t="n">
+      <c r="V13" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="U13" s="7" t="n">
+      <c r="W13" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="V13" s="7" t="n">
+      <c r="X13" s="7" t="n">
         <v>52</v>
+      </c>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>Finished_Bacardi</t>
+        </is>
+      </c>
+      <c r="Z13" s="7" t="inlineStr">
+        <is>
+          <t>Serve_Bacardi</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -3205,22 +3613,42 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>보드카 4oz, 쿠앵트로 1.5oz, 크랜베리주스 3oz, 라임즙 1.5oz를 셰이킹해 칵테일 잔에 따른다. 레몬 슬라이스를 올린다.</t>
+        </is>
+      </c>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>Shake 4oz vodka, 1.5oz cointreau, 3oz cranberry juice, and 1.5oz lime juice, then strain into a cocktail glass. Add a lemon slice.</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="S14" t="n">
+      <c r="U14" t="n">
         <v>5</v>
       </c>
-      <c r="T14" t="n">
+      <c r="V14" t="n">
         <v>2</v>
       </c>
-      <c r="U14" t="n">
+      <c r="W14" t="n">
         <v>8</v>
       </c>
-      <c r="V14" t="n">
+      <c r="X14" t="n">
         <v>60</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Finished_Cosmopolitan</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Serve_Cosmopolitan</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -3285,22 +3713,42 @@
       <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr"/>
       <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr">
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>데킬라 3.5oz, 트리플섹 2oz, 레몬즙 1.5oz를 셰이킹해 칵테일 잔에 따른다. 라임 웨지를 걸친다.</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr">
+        <is>
+          <t>Shake 3.5oz tequila, 2oz triple sec, and 1.5oz lemon juice, then strain into a cocktail glass. Garnish with a lime wedge.</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S15" s="7" t="n">
+      <c r="U15" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="T15" s="7" t="n">
+      <c r="V15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="U15" s="7" t="n">
+      <c r="W15" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="V15" s="7" t="n">
+      <c r="X15" s="7" t="n">
         <v>52</v>
+      </c>
+      <c r="Y15" s="7" t="inlineStr">
+        <is>
+          <t>Finished_Margarita</t>
+        </is>
+      </c>
+      <c r="Z15" s="7" t="inlineStr">
+        <is>
+          <t>Serve_Margarita</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -3361,22 +3809,42 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>진 40ml, 트리플섹 30ml, 레몬즙 20ml를 셰이킹해 칵테일 잔에 따른다.</t>
+        </is>
+      </c>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>Shake 40ml gin, 30ml triple sec, and 20ml lemon juice, then strain into a cocktail glass.</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S16" t="n">
+      <c r="U16" t="n">
         <v>4</v>
       </c>
-      <c r="T16" t="n">
+      <c r="V16" t="n">
         <v>6</v>
       </c>
-      <c r="U16" t="n">
+      <c r="W16" t="n">
         <v>7</v>
       </c>
-      <c r="V16" t="n">
+      <c r="X16" t="n">
         <v>52</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Finished_WhiteLady</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Serve_WhiteLady</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3437,22 +3905,42 @@
       <c r="O17" s="7" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr"/>
       <c r="Q17" s="7" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr">
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>온더락 잔에 칼루아 1.5oz를 붓고 우유 0.75oz를 위에 얹듯 천천히 따른다.</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>Pour 1.5oz kahlua into a rocks glass, then layer 0.75oz milk slowly on top.</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="S17" s="7" t="n">
+      <c r="U17" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="T17" s="7" t="n">
+      <c r="V17" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="U17" s="7" t="n">
+      <c r="W17" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="V17" s="7" t="n">
+      <c r="X17" s="7" t="n">
         <v>44</v>
+      </c>
+      <c r="Y17" s="7" t="inlineStr">
+        <is>
+          <t>Finished_KahluaMilk</t>
+        </is>
+      </c>
+      <c r="Z17" s="7" t="inlineStr">
+        <is>
+          <t>Serve_KahluaMilk</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -3517,32 +4005,301 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>진 2oz, 벌꿀 원액 0.75oz, 레몬즙 0.75oz를 셰이킹해 칵테일 잔에 따른다. 레몬 슬라이스를 올린다.</t>
+        </is>
+      </c>
+      <c r="S18" s="6" t="inlineStr">
+        <is>
+          <t>Shake 2oz gin, 0.75oz honey syrup, and 0.75oz lemon juice, then strain into a cocktail glass. Add a lemon slice.</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="S18" t="n">
+      <c r="U18" t="n">
         <v>4</v>
       </c>
-      <c r="T18" t="n">
+      <c r="V18" t="n">
         <v>99</v>
       </c>
-      <c r="U18" t="n">
+      <c r="W18" t="n">
         <v>7</v>
       </c>
-      <c r="V18" t="n">
+      <c r="X18" t="n">
         <v>52</v>
       </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Finished_BeesKnees</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Serve_BeesKnees</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V18"/>
+  <autoFilter ref="A1:Z18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>tag_ko</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>tag_en</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>가벼운</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>저도수·부담 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>달콤한</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Sweet</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>독한</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>고도수</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>묵직한</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>바디감</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>부드러운</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Smooth</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>비밀</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>비밀 레시피 계열</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>상큼한</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>시트러스</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>새콤한</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tangy</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>씁쓸한</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bitter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>알싸한</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Spicy</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>진저 계열의 톡 쏘는 맛</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>우아한</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elegant</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>청량한</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>탄산감</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>클래식</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Classic</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>화사한</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Bright</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
@@ -4747,7 +5504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
@@ -6710,7 +7467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
@@ -6928,7 +7685,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -7180,14 +7937,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00ED7D31"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -7855,148 +8612,87 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>order_bark_gap_sec</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>1.5</v>
+          <t>sfx_serve</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>SFX_glass_slide</t>
+        </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>주문 대사 사이의 텀 — ask_order→order_think→order 순서로 재생할 때, 앞 대사 타이핑이 끝나고 다음 대사까지 기다리는 초 [가안]</t>
+          <t>제공 컷씬 공용 사운드(잔 미는 소리) — 구엔진 이식, 전 칵테일 공용</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>street_typing_interval_ms</t>
+          <t>order_bark_gap_sec</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50</v>
+        <v>1.5</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>거리 말풍선 타이핑 문자당 간격(ms) — 바(typing_interval_ms)와 별도 튜닝</t>
+          <t>주문 대사 사이의 텀 — ask_order→order_think→order 순서로 재생할 때, 앞 대사 타이핑이 끝나고 다음 대사까지 기다리는 초 [가안]</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
+          <t>street_typing_interval_ms</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>거리 말풍선 타이핑 문자당 간격(ms) — 바(typing_interval_ms)와 별도 튜닝</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>street_auto_next_delay_sec</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B36" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>auto 재생 대사 — 타이핑 종료 후 다음 대사까지 텀</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D35"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00ED7D31"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>grade</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>min_pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>excellent</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>decent</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>poor</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>sewage</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:D36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -8013,7 +8709,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8024,7 +8720,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>revenue_mult</t>
+          <t>min_pct</t>
         </is>
       </c>
     </row>
@@ -8035,7 +8731,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.2</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -8045,7 +8741,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
@@ -8055,7 +8751,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -8065,7 +8761,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>0.3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -8075,7 +8771,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>